<commit_message>
updates for TT supplier
</commit_message>
<xml_diff>
--- a/data/ready_stocks/tt-ozon-stocks-updated.xlsx
+++ b/data/ready_stocks/tt-ozon-stocks-updated.xlsx
@@ -774,7 +774,7 @@
         <v/>
       </c>
       <c r="D27">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -802,7 +802,7 @@
         <v/>
       </c>
       <c r="D29">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -844,7 +844,7 @@
         <v/>
       </c>
       <c r="D32">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -872,7 +872,7 @@
         <v/>
       </c>
       <c r="D34">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -886,7 +886,7 @@
         <v/>
       </c>
       <c r="D35">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -900,7 +900,7 @@
         <v/>
       </c>
       <c r="D36">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -914,7 +914,7 @@
         <v/>
       </c>
       <c r="D37">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>